<commit_message>
docs: drop MongoDB from the roadmap and project context
MongoDB is no longer part of the stack: the Trustpilot reviews and the
SDV synthetic data go to PostgreSQL, with JSONB for the semi-structured
part, as listed in the updated technology comparison.

- monthly roadmap and both spreadsheets: P3 now covers JSONB storage of
  the reviews instead of a MongoDB role, P4 loads reviews and SDV data
  into PostgreSQL instead of linking Postgres and Mongo
- the P2 tech watch keeps the PostgreSQL vs MongoDB comparison, now
  framed as the justification for choosing PostgreSQL
- CLAUDE.md context: storage line updated, scraping (BeautifulSoup) and
  SDV mentioned

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Roadmap/roadmap_churn_2026-2027_v2.xlsx
+++ b/Roadmap/roadmap_churn_2026-2027_v2.xlsx
@@ -1263,7 +1263,7 @@
       <c r="A23" s="16" t="n"/>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>MPD PostgreSQL Bronze/Silver/Gold + rôle MongoDB</t>
+          <t>MPD PostgreSQL Bronze/Silver/Gold + stockage JSONB des avis</t>
         </is>
       </c>
       <c r="C23" s="19" t="n"/>
@@ -1451,7 +1451,7 @@
       <c r="A31" s="16" t="n"/>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>Nettoyage qualité + bases Postgres / Mongo reliées</t>
+          <t>Nettoyage qualité + avis Trustpilot / SDV dans PostgreSQL (JSONB)</t>
         </is>
       </c>
       <c r="C31" s="19" t="n"/>

</xml_diff>